<commit_message>
Calibrated and updated power sector data
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Models\US\Models\eps-us\InputData\elec\BBNPPTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED5C7C3-C6DD-4CC0-A75D-D5DA17DC76DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703EACAA-B4B9-4932-BFEF-1DCFA13430D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3900" windowWidth="38865" windowHeight="17235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6825" yWindow="4485" windowWidth="17280" windowHeight="10005" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Source:</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>and the construction time for new or modified plants.</t>
+  </si>
+  <si>
+    <t>2026-08-21 power-sector calibration (cal9): endogenous builds banned through 2030 for hard coal, lignite, nuclear, and SMR - lead-time convention (multi-year construction means nothing not already in the pipeline can come online before ~2030; the pipeline enters via the mandated schedule). Post-2030 the economic build channel reopens.</t>
+  </si>
+  <si>
+    <t>2026-09-04 start-year convention (matches eps-us, INITIAL TIME 2025 / vintages end 2024 / BPMCCS 2025 = first-year builds / BBNPPTY bans all sources through the last historical year): all sources banned from endogenous builds through 2025, the last year with actual installation data in BPMCCS (설비현황_19~25). Historical capacity therefore comes only from start-year vintages (through 2020) plus the mandated schedule. Lead-time bans for coal/lignite/nuclear/SMR through 2030 unchanged.</t>
   </si>
 </sst>
 </file>
@@ -523,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="60.85546875" customWidth="1"/>
@@ -590,6 +596,16 @@
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -719,16 +735,16 @@
         <v>1</v>
       </c>
       <c r="E2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="5">
         <v>1</v>
@@ -814,10 +830,10 @@
         <v>1</v>
       </c>
       <c r="E3" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="5">
         <v>0</v>
@@ -909,10 +925,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="5">
         <v>0</v>
@@ -1004,25 +1020,25 @@
         <v>1</v>
       </c>
       <c r="E5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="5">
         <v>0</v>
@@ -1099,10 +1115,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="5">
         <v>0</v>
@@ -1194,10 +1210,10 @@
         <v>1</v>
       </c>
       <c r="E7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="5">
         <v>0</v>
@@ -1289,10 +1305,10 @@
         <v>1</v>
       </c>
       <c r="E8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="5">
         <v>0</v>
@@ -1384,10 +1400,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="5">
         <v>0</v>
@@ -1479,10 +1495,10 @@
         <v>1</v>
       </c>
       <c r="E10" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="5">
         <v>0</v>
@@ -1574,10 +1590,10 @@
         <v>1</v>
       </c>
       <c r="E11" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="5">
         <v>0</v>
@@ -1669,10 +1685,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="5">
         <v>0</v>
@@ -1764,10 +1780,10 @@
         <v>1</v>
       </c>
       <c r="E13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="5">
         <v>0</v>
@@ -1859,16 +1875,16 @@
         <v>1</v>
       </c>
       <c r="E14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="5">
         <v>1</v>
@@ -1954,10 +1970,10 @@
         <v>1</v>
       </c>
       <c r="E15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="5">
         <v>0</v>
@@ -2049,10 +2065,10 @@
         <v>1</v>
       </c>
       <c r="E16" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="5">
         <v>0</v>
@@ -2144,10 +2160,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="5">
         <v>0</v>
@@ -2239,10 +2255,10 @@
         <v>1</v>
       </c>
       <c r="E18" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="5">
         <v>0</v>
@@ -2714,25 +2730,25 @@
         <v>1</v>
       </c>
       <c r="E23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" s="5">
         <v>0</v>
@@ -2809,10 +2825,10 @@
         <v>1</v>
       </c>
       <c r="E24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="5">
         <v>0</v>
@@ -2904,10 +2920,10 @@
         <v>1</v>
       </c>
       <c r="E25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="5">
         <v>0</v>
@@ -2992,6 +3008,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -3135,7 +3157,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3144,20 +3166,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{971C8F4A-E10E-4C19-844B-3416D802FA23}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAC2D09F-B9CA-4F44-B9DD-E131E48950C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3F51D06-EFCE-4C0B-BB57-11FFF6362EB6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{971C8F4A-E10E-4C19-844B-3416D802FA23}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAC2D09F-B9CA-4F44-B9DD-E131E48950C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3F51D06-EFCE-4C0B-BB57-11FFF6362EB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>